<commit_message>
Competencia, Estudio de Mercado y Ajustes al Marco Teorico
</commit_message>
<xml_diff>
--- a/Archivos/Cronograma.xlsx
+++ b/Archivos/Cronograma.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\OneDrive\Escritorio\TexProyecto\Archivos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\OneDrive\Escritorio\GitHubProyecto\anteproyecto\Archivos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39BA920B-B13B-46B0-AB2C-BFA85FCBC2E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D04368F-FC41-4F9F-81B9-606BD0A011B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15840" xr2:uid="{1AE7592A-28E1-42CE-90E1-271931B8FD3D}"/>
   </bookViews>
@@ -124,22 +124,22 @@
     <t>Semanas</t>
   </si>
   <si>
-    <t>Agosto</t>
-  </si>
-  <si>
-    <t>Septiembre</t>
-  </si>
-  <si>
-    <t>Octubre</t>
-  </si>
-  <si>
-    <t>Noviembre</t>
-  </si>
-  <si>
-    <t>Diciembre</t>
-  </si>
-  <si>
-    <t>Julio</t>
+    <t>Febrero</t>
+  </si>
+  <si>
+    <t>Marzo</t>
+  </si>
+  <si>
+    <t>Abril</t>
+  </si>
+  <si>
+    <t>Mayo</t>
+  </si>
+  <si>
+    <t>Junio</t>
+  </si>
+  <si>
+    <t>Enero</t>
   </si>
 </sst>
 </file>
@@ -313,12 +313,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -326,6 +320,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -668,41 +668,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A1" s="16"/>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-      <c r="N1" s="16"/>
-      <c r="O1" s="16"/>
-      <c r="P1" s="16"/>
-      <c r="Q1" s="16"/>
-      <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
-      <c r="T1" s="16"/>
-      <c r="U1" s="16"/>
-      <c r="V1" s="16"/>
-      <c r="W1" s="16"/>
-      <c r="X1" s="16"/>
-      <c r="Y1" s="16"/>
-      <c r="Z1" s="16"/>
-      <c r="AA1" s="16"/>
-      <c r="AB1" s="16"/>
+      <c r="A1" s="14"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="G1" s="14"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
+      <c r="T1" s="14"/>
+      <c r="U1" s="14"/>
+      <c r="V1" s="14"/>
+      <c r="W1" s="14"/>
+      <c r="X1" s="14"/>
+      <c r="Y1" s="14"/>
+      <c r="Z1" s="14"/>
+      <c r="AA1" s="14"/>
+      <c r="AB1" s="14"/>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A2" s="16"/>
-      <c r="B2" s="18" t="s">
+      <c r="A2" s="14"/>
+      <c r="B2" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="16" t="s">
         <v>25</v>
       </c>
       <c r="D2" s="6">
@@ -777,30 +777,30 @@
       <c r="AA2" s="9">
         <v>24</v>
       </c>
-      <c r="AB2" s="16"/>
+      <c r="AB2" s="14"/>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A3" s="16"/>
-      <c r="B3" s="18"/>
-      <c r="C3" s="18"/>
-      <c r="D3" s="14" t="s">
+      <c r="A3" s="14"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="15" t="s">
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="14" t="s">
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
+      <c r="M3" s="17"/>
+      <c r="N3" s="17"/>
+      <c r="O3" s="17"/>
       <c r="P3" s="19" t="s">
         <v>28</v>
       </c>
@@ -819,47 +819,47 @@
       </c>
       <c r="Z3" s="20"/>
       <c r="AA3" s="21"/>
-      <c r="AB3" s="16"/>
+      <c r="AB3" s="14"/>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A4" s="16"/>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="16"/>
+      <c r="C4" s="16"/>
       <c r="D4" s="6">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E4" s="6">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F4" s="6">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G4" s="6">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H4" s="9">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I4" s="9">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J4" s="9">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K4" s="9">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="L4" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M4" s="6">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N4" s="6">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="O4" s="6">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="P4" s="9">
         <v>1</v>
@@ -877,30 +877,30 @@
         <v>29</v>
       </c>
       <c r="U4" s="7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="V4" s="7">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="W4" s="7">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="X4" s="7">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Y4" s="9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="Z4" s="9">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="AA4" s="9">
-        <v>19</v>
-      </c>
-      <c r="AB4" s="16"/>
+        <v>17</v>
+      </c>
+      <c r="AB4" s="14"/>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A5" s="16"/>
+      <c r="A5" s="14"/>
       <c r="B5" s="3" t="s">
         <v>0</v>
       </c>
@@ -931,10 +931,10 @@
       <c r="Y5" s="5"/>
       <c r="Z5" s="5"/>
       <c r="AA5" s="5"/>
-      <c r="AB5" s="16"/>
+      <c r="AB5" s="14"/>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A6" s="16"/>
+      <c r="A6" s="14"/>
       <c r="B6" s="1" t="s">
         <v>1</v>
       </c>
@@ -965,10 +965,10 @@
       <c r="Y6" s="10"/>
       <c r="Z6" s="10"/>
       <c r="AA6" s="10"/>
-      <c r="AB6" s="16"/>
+      <c r="AB6" s="14"/>
     </row>
     <row r="7" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A7" s="16"/>
+      <c r="A7" s="14"/>
       <c r="B7" s="1" t="s">
         <v>2</v>
       </c>
@@ -999,10 +999,10 @@
       <c r="Y7" s="10"/>
       <c r="Z7" s="10"/>
       <c r="AA7" s="10"/>
-      <c r="AB7" s="16"/>
+      <c r="AB7" s="14"/>
     </row>
     <row r="8" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A8" s="16"/>
+      <c r="A8" s="14"/>
       <c r="B8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1033,10 +1033,10 @@
       <c r="Y8" s="10"/>
       <c r="Z8" s="10"/>
       <c r="AA8" s="10"/>
-      <c r="AB8" s="16"/>
+      <c r="AB8" s="14"/>
     </row>
     <row r="9" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="16"/>
+      <c r="A9" s="14"/>
       <c r="B9" s="2" t="s">
         <v>17</v>
       </c>
@@ -1067,10 +1067,10 @@
       <c r="Y9" s="10"/>
       <c r="Z9" s="10"/>
       <c r="AA9" s="10"/>
-      <c r="AB9" s="16"/>
+      <c r="AB9" s="14"/>
     </row>
     <row r="10" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
+      <c r="A10" s="14"/>
       <c r="B10" s="2" t="s">
         <v>18</v>
       </c>
@@ -1101,10 +1101,10 @@
       <c r="Y10" s="10"/>
       <c r="Z10" s="10"/>
       <c r="AA10" s="10"/>
-      <c r="AB10" s="16"/>
+      <c r="AB10" s="14"/>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A11" s="16"/>
+      <c r="A11" s="14"/>
       <c r="B11" s="3" t="s">
         <v>4</v>
       </c>
@@ -1135,10 +1135,10 @@
       <c r="Y11" s="5"/>
       <c r="Z11" s="5"/>
       <c r="AA11" s="5"/>
-      <c r="AB11" s="16"/>
+      <c r="AB11" s="14"/>
     </row>
     <row r="12" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16"/>
+      <c r="A12" s="14"/>
       <c r="B12" s="2" t="s">
         <v>19</v>
       </c>
@@ -1169,10 +1169,10 @@
       <c r="Y12" s="10"/>
       <c r="Z12" s="10"/>
       <c r="AA12" s="10"/>
-      <c r="AB12" s="16"/>
+      <c r="AB12" s="14"/>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
+      <c r="A13" s="14"/>
       <c r="B13" s="1" t="s">
         <v>5</v>
       </c>
@@ -1203,10 +1203,10 @@
       <c r="Y13" s="10"/>
       <c r="Z13" s="10"/>
       <c r="AA13" s="10"/>
-      <c r="AB13" s="16"/>
+      <c r="AB13" s="14"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A14" s="16"/>
+      <c r="A14" s="14"/>
       <c r="B14" s="1" t="s">
         <v>6</v>
       </c>
@@ -1237,10 +1237,10 @@
       <c r="Y14" s="10"/>
       <c r="Z14" s="10"/>
       <c r="AA14" s="10"/>
-      <c r="AB14" s="16"/>
+      <c r="AB14" s="14"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A15" s="16"/>
+      <c r="A15" s="14"/>
       <c r="B15" s="3" t="s">
         <v>7</v>
       </c>
@@ -1271,10 +1271,10 @@
       <c r="Y15" s="5"/>
       <c r="Z15" s="5"/>
       <c r="AA15" s="5"/>
-      <c r="AB15" s="16"/>
+      <c r="AB15" s="14"/>
     </row>
     <row r="16" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="16"/>
+      <c r="A16" s="14"/>
       <c r="B16" s="2" t="s">
         <v>20</v>
       </c>
@@ -1305,10 +1305,10 @@
       <c r="Y16" s="10"/>
       <c r="Z16" s="10"/>
       <c r="AA16" s="10"/>
-      <c r="AB16" s="16"/>
+      <c r="AB16" s="14"/>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A17" s="16"/>
+      <c r="A17" s="14"/>
       <c r="B17" s="1" t="s">
         <v>8</v>
       </c>
@@ -1339,10 +1339,10 @@
       <c r="Y17" s="10"/>
       <c r="Z17" s="10"/>
       <c r="AA17" s="10"/>
-      <c r="AB17" s="16"/>
+      <c r="AB17" s="14"/>
     </row>
     <row r="18" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A18" s="16"/>
+      <c r="A18" s="14"/>
       <c r="B18" s="1" t="s">
         <v>16</v>
       </c>
@@ -1373,10 +1373,10 @@
       <c r="Y18" s="10"/>
       <c r="Z18" s="10"/>
       <c r="AA18" s="10"/>
-      <c r="AB18" s="16"/>
+      <c r="AB18" s="14"/>
     </row>
     <row r="19" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A19" s="16"/>
+      <c r="A19" s="14"/>
       <c r="B19" s="1" t="s">
         <v>9</v>
       </c>
@@ -1407,10 +1407,10 @@
       <c r="Y19" s="10"/>
       <c r="Z19" s="10"/>
       <c r="AA19" s="10"/>
-      <c r="AB19" s="16"/>
+      <c r="AB19" s="14"/>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A20" s="16"/>
+      <c r="A20" s="14"/>
       <c r="B20" s="3" t="s">
         <v>10</v>
       </c>
@@ -1441,10 +1441,10 @@
       <c r="Y20" s="5"/>
       <c r="Z20" s="5"/>
       <c r="AA20" s="5"/>
-      <c r="AB20" s="16"/>
+      <c r="AB20" s="14"/>
     </row>
     <row r="21" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="16"/>
+      <c r="A21" s="14"/>
       <c r="B21" s="2" t="s">
         <v>21</v>
       </c>
@@ -1475,10 +1475,10 @@
       <c r="Y21" s="10"/>
       <c r="Z21" s="10"/>
       <c r="AA21" s="10"/>
-      <c r="AB21" s="16"/>
+      <c r="AB21" s="14"/>
     </row>
     <row r="22" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="16"/>
+      <c r="A22" s="14"/>
       <c r="B22" s="2" t="s">
         <v>22</v>
       </c>
@@ -1509,10 +1509,10 @@
       <c r="Y22" s="10"/>
       <c r="Z22" s="10"/>
       <c r="AA22" s="10"/>
-      <c r="AB22" s="16"/>
+      <c r="AB22" s="14"/>
     </row>
     <row r="23" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="16"/>
+      <c r="A23" s="14"/>
       <c r="B23" s="2" t="s">
         <v>23</v>
       </c>
@@ -1543,10 +1543,10 @@
       <c r="Y23" s="10"/>
       <c r="Z23" s="10"/>
       <c r="AA23" s="10"/>
-      <c r="AB23" s="16"/>
+      <c r="AB23" s="14"/>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A24" s="16"/>
+      <c r="A24" s="14"/>
       <c r="B24" s="1" t="s">
         <v>11</v>
       </c>
@@ -1577,10 +1577,10 @@
       <c r="Y24" s="10"/>
       <c r="Z24" s="10"/>
       <c r="AA24" s="10"/>
-      <c r="AB24" s="16"/>
+      <c r="AB24" s="14"/>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A25" s="16"/>
+      <c r="A25" s="14"/>
       <c r="B25" s="1" t="s">
         <v>12</v>
       </c>
@@ -1611,10 +1611,10 @@
       <c r="Y25" s="10"/>
       <c r="Z25" s="10"/>
       <c r="AA25" s="10"/>
-      <c r="AB25" s="16"/>
+      <c r="AB25" s="14"/>
     </row>
     <row r="26" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A26" s="16"/>
+      <c r="A26" s="14"/>
       <c r="B26" s="1" t="s">
         <v>13</v>
       </c>
@@ -1645,10 +1645,10 @@
       <c r="Y26" s="10"/>
       <c r="Z26" s="10"/>
       <c r="AA26" s="10"/>
-      <c r="AB26" s="16"/>
+      <c r="AB26" s="14"/>
     </row>
     <row r="27" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A27" s="16"/>
+      <c r="A27" s="14"/>
       <c r="B27" s="1" t="s">
         <v>14</v>
       </c>
@@ -1679,10 +1679,10 @@
       <c r="Y27" s="10"/>
       <c r="Z27" s="10"/>
       <c r="AA27" s="10"/>
-      <c r="AB27" s="16"/>
+      <c r="AB27" s="14"/>
     </row>
     <row r="28" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A28" s="16"/>
+      <c r="A28" s="14"/>
       <c r="B28" s="1" t="s">
         <v>15</v>
       </c>
@@ -1713,217 +1713,217 @@
       <c r="Y28" s="10"/>
       <c r="Z28" s="10"/>
       <c r="AA28" s="10"/>
-      <c r="AB28" s="16"/>
+      <c r="AB28" s="14"/>
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A29" s="16"/>
-      <c r="B29" s="17"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
-      <c r="E29" s="17"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
-      <c r="J29" s="17"/>
-      <c r="K29" s="17"/>
-      <c r="L29" s="17"/>
-      <c r="M29" s="17"/>
-      <c r="N29" s="17"/>
-      <c r="O29" s="17"/>
-      <c r="P29" s="17"/>
-      <c r="Q29" s="17"/>
-      <c r="R29" s="17"/>
-      <c r="S29" s="17"/>
-      <c r="T29" s="17"/>
-      <c r="U29" s="17"/>
-      <c r="V29" s="17"/>
-      <c r="W29" s="17"/>
-      <c r="X29" s="17"/>
-      <c r="Y29" s="17"/>
-      <c r="Z29" s="17"/>
-      <c r="AA29" s="17"/>
-      <c r="AB29" s="16"/>
+      <c r="A29" s="14"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="15"/>
+      <c r="K29" s="15"/>
+      <c r="L29" s="15"/>
+      <c r="M29" s="15"/>
+      <c r="N29" s="15"/>
+      <c r="O29" s="15"/>
+      <c r="P29" s="15"/>
+      <c r="Q29" s="15"/>
+      <c r="R29" s="15"/>
+      <c r="S29" s="15"/>
+      <c r="T29" s="15"/>
+      <c r="U29" s="15"/>
+      <c r="V29" s="15"/>
+      <c r="W29" s="15"/>
+      <c r="X29" s="15"/>
+      <c r="Y29" s="15"/>
+      <c r="Z29" s="15"/>
+      <c r="AA29" s="15"/>
+      <c r="AB29" s="14"/>
     </row>
     <row r="30" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A30" s="16"/>
-      <c r="B30" s="16"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
-      <c r="G30" s="16"/>
-      <c r="H30" s="16"/>
-      <c r="I30" s="16"/>
-      <c r="J30" s="16"/>
-      <c r="K30" s="16"/>
-      <c r="L30" s="16"/>
-      <c r="M30" s="16"/>
-      <c r="N30" s="16"/>
-      <c r="O30" s="16"/>
-      <c r="P30" s="16"/>
-      <c r="Q30" s="16"/>
-      <c r="R30" s="16"/>
-      <c r="S30" s="16"/>
-      <c r="T30" s="16"/>
-      <c r="U30" s="16"/>
-      <c r="V30" s="16"/>
-      <c r="W30" s="16"/>
-      <c r="X30" s="16"/>
-      <c r="Y30" s="16"/>
-      <c r="Z30" s="16"/>
-      <c r="AA30" s="16"/>
-      <c r="AB30" s="16"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="14"/>
+      <c r="J30" s="14"/>
+      <c r="K30" s="14"/>
+      <c r="L30" s="14"/>
+      <c r="M30" s="14"/>
+      <c r="N30" s="14"/>
+      <c r="O30" s="14"/>
+      <c r="P30" s="14"/>
+      <c r="Q30" s="14"/>
+      <c r="R30" s="14"/>
+      <c r="S30" s="14"/>
+      <c r="T30" s="14"/>
+      <c r="U30" s="14"/>
+      <c r="V30" s="14"/>
+      <c r="W30" s="14"/>
+      <c r="X30" s="14"/>
+      <c r="Y30" s="14"/>
+      <c r="Z30" s="14"/>
+      <c r="AA30" s="14"/>
+      <c r="AB30" s="14"/>
     </row>
     <row r="31" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A31" s="16"/>
-      <c r="B31" s="16"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16"/>
-      <c r="F31" s="16"/>
-      <c r="G31" s="16"/>
-      <c r="H31" s="16"/>
-      <c r="I31" s="16"/>
-      <c r="J31" s="16"/>
-      <c r="K31" s="16"/>
-      <c r="L31" s="16"/>
-      <c r="M31" s="16"/>
-      <c r="N31" s="16"/>
-      <c r="O31" s="16"/>
-      <c r="P31" s="16"/>
-      <c r="Q31" s="16"/>
-      <c r="R31" s="16"/>
-      <c r="S31" s="16"/>
-      <c r="T31" s="16"/>
-      <c r="U31" s="16"/>
-      <c r="V31" s="16"/>
-      <c r="W31" s="16"/>
-      <c r="X31" s="16"/>
-      <c r="Y31" s="16"/>
-      <c r="Z31" s="16"/>
-      <c r="AA31" s="16"/>
-      <c r="AB31" s="16"/>
+      <c r="A31" s="14"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="14"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="14"/>
+      <c r="L31" s="14"/>
+      <c r="M31" s="14"/>
+      <c r="N31" s="14"/>
+      <c r="O31" s="14"/>
+      <c r="P31" s="14"/>
+      <c r="Q31" s="14"/>
+      <c r="R31" s="14"/>
+      <c r="S31" s="14"/>
+      <c r="T31" s="14"/>
+      <c r="U31" s="14"/>
+      <c r="V31" s="14"/>
+      <c r="W31" s="14"/>
+      <c r="X31" s="14"/>
+      <c r="Y31" s="14"/>
+      <c r="Z31" s="14"/>
+      <c r="AA31" s="14"/>
+      <c r="AB31" s="14"/>
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A32" s="16"/>
-      <c r="B32" s="16"/>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="16"/>
-      <c r="F32" s="16"/>
-      <c r="G32" s="16"/>
-      <c r="H32" s="16"/>
-      <c r="I32" s="16"/>
-      <c r="J32" s="16"/>
-      <c r="K32" s="16"/>
-      <c r="L32" s="16"/>
-      <c r="M32" s="16"/>
-      <c r="N32" s="16"/>
-      <c r="O32" s="16"/>
-      <c r="P32" s="16"/>
-      <c r="Q32" s="16"/>
-      <c r="R32" s="16"/>
-      <c r="S32" s="16"/>
-      <c r="T32" s="16"/>
-      <c r="U32" s="16"/>
-      <c r="V32" s="16"/>
-      <c r="W32" s="16"/>
-      <c r="X32" s="16"/>
-      <c r="Y32" s="16"/>
-      <c r="Z32" s="16"/>
-      <c r="AA32" s="16"/>
-      <c r="AB32" s="16"/>
+      <c r="A32" s="14"/>
+      <c r="B32" s="14"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
+      <c r="I32" s="14"/>
+      <c r="J32" s="14"/>
+      <c r="K32" s="14"/>
+      <c r="L32" s="14"/>
+      <c r="M32" s="14"/>
+      <c r="N32" s="14"/>
+      <c r="O32" s="14"/>
+      <c r="P32" s="14"/>
+      <c r="Q32" s="14"/>
+      <c r="R32" s="14"/>
+      <c r="S32" s="14"/>
+      <c r="T32" s="14"/>
+      <c r="U32" s="14"/>
+      <c r="V32" s="14"/>
+      <c r="W32" s="14"/>
+      <c r="X32" s="14"/>
+      <c r="Y32" s="14"/>
+      <c r="Z32" s="14"/>
+      <c r="AA32" s="14"/>
+      <c r="AB32" s="14"/>
     </row>
     <row r="33" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A33" s="16"/>
-      <c r="B33" s="16"/>
-      <c r="C33" s="16"/>
-      <c r="D33" s="16"/>
-      <c r="E33" s="16"/>
-      <c r="F33" s="16"/>
-      <c r="G33" s="16"/>
-      <c r="H33" s="16"/>
-      <c r="I33" s="16"/>
-      <c r="J33" s="16"/>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
-      <c r="M33" s="16"/>
-      <c r="N33" s="16"/>
-      <c r="O33" s="16"/>
-      <c r="P33" s="16"/>
-      <c r="Q33" s="16"/>
-      <c r="R33" s="16"/>
-      <c r="S33" s="16"/>
-      <c r="T33" s="16"/>
-      <c r="U33" s="16"/>
-      <c r="V33" s="16"/>
-      <c r="W33" s="16"/>
-      <c r="X33" s="16"/>
-      <c r="Y33" s="16"/>
-      <c r="Z33" s="16"/>
-      <c r="AA33" s="16"/>
-      <c r="AB33" s="16"/>
+      <c r="A33" s="14"/>
+      <c r="B33" s="14"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+      <c r="I33" s="14"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="14"/>
+      <c r="L33" s="14"/>
+      <c r="M33" s="14"/>
+      <c r="N33" s="14"/>
+      <c r="O33" s="14"/>
+      <c r="P33" s="14"/>
+      <c r="Q33" s="14"/>
+      <c r="R33" s="14"/>
+      <c r="S33" s="14"/>
+      <c r="T33" s="14"/>
+      <c r="U33" s="14"/>
+      <c r="V33" s="14"/>
+      <c r="W33" s="14"/>
+      <c r="X33" s="14"/>
+      <c r="Y33" s="14"/>
+      <c r="Z33" s="14"/>
+      <c r="AA33" s="14"/>
+      <c r="AB33" s="14"/>
     </row>
     <row r="34" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A34" s="16"/>
-      <c r="B34" s="16"/>
-      <c r="C34" s="16"/>
-      <c r="D34" s="16"/>
-      <c r="E34" s="16"/>
-      <c r="F34" s="16"/>
-      <c r="G34" s="16"/>
-      <c r="H34" s="16"/>
-      <c r="I34" s="16"/>
-      <c r="J34" s="16"/>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
-      <c r="N34" s="16"/>
-      <c r="O34" s="16"/>
-      <c r="P34" s="16"/>
-      <c r="Q34" s="16"/>
-      <c r="R34" s="16"/>
-      <c r="S34" s="16"/>
-      <c r="T34" s="16"/>
-      <c r="U34" s="16"/>
-      <c r="V34" s="16"/>
-      <c r="W34" s="16"/>
-      <c r="X34" s="16"/>
-      <c r="Y34" s="16"/>
-      <c r="Z34" s="16"/>
-      <c r="AA34" s="16"/>
-      <c r="AB34" s="16"/>
+      <c r="A34" s="14"/>
+      <c r="B34" s="14"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="14"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="14"/>
+      <c r="L34" s="14"/>
+      <c r="M34" s="14"/>
+      <c r="N34" s="14"/>
+      <c r="O34" s="14"/>
+      <c r="P34" s="14"/>
+      <c r="Q34" s="14"/>
+      <c r="R34" s="14"/>
+      <c r="S34" s="14"/>
+      <c r="T34" s="14"/>
+      <c r="U34" s="14"/>
+      <c r="V34" s="14"/>
+      <c r="W34" s="14"/>
+      <c r="X34" s="14"/>
+      <c r="Y34" s="14"/>
+      <c r="Z34" s="14"/>
+      <c r="AA34" s="14"/>
+      <c r="AB34" s="14"/>
     </row>
     <row r="35" spans="1:28" x14ac:dyDescent="0.25">
-      <c r="A35" s="16"/>
-      <c r="B35" s="16"/>
-      <c r="C35" s="16"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="16"/>
-      <c r="F35" s="16"/>
-      <c r="G35" s="16"/>
-      <c r="H35" s="16"/>
-      <c r="I35" s="16"/>
-      <c r="J35" s="16"/>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="16"/>
-      <c r="O35" s="16"/>
-      <c r="P35" s="16"/>
-      <c r="Q35" s="16"/>
-      <c r="R35" s="16"/>
-      <c r="S35" s="16"/>
-      <c r="T35" s="16"/>
-      <c r="U35" s="16"/>
-      <c r="V35" s="16"/>
-      <c r="W35" s="16"/>
-      <c r="X35" s="16"/>
-      <c r="Y35" s="16"/>
-      <c r="Z35" s="16"/>
-      <c r="AA35" s="16"/>
-      <c r="AB35" s="16"/>
+      <c r="A35" s="14"/>
+      <c r="B35" s="14"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
+      <c r="I35" s="14"/>
+      <c r="J35" s="14"/>
+      <c r="K35" s="14"/>
+      <c r="L35" s="14"/>
+      <c r="M35" s="14"/>
+      <c r="N35" s="14"/>
+      <c r="O35" s="14"/>
+      <c r="P35" s="14"/>
+      <c r="Q35" s="14"/>
+      <c r="R35" s="14"/>
+      <c r="S35" s="14"/>
+      <c r="T35" s="14"/>
+      <c r="U35" s="14"/>
+      <c r="V35" s="14"/>
+      <c r="W35" s="14"/>
+      <c r="X35" s="14"/>
+      <c r="Y35" s="14"/>
+      <c r="Z35" s="14"/>
+      <c r="AA35" s="14"/>
+      <c r="AB35" s="14"/>
     </row>
     <row r="36" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A36" s="13"/>

</xml_diff>